<commit_message>
Fix real gaps: add CSV export to The Ledger, add real profit-factor/largest-win-loss/equity-curve to the Excel journal template, add 3 fundamentals lessons (pips/lots/spread, leverage/margin, order types) to close the Learn Everything content gap
</commit_message>
<xml_diff>
--- a/files/trading-journal-template.xlsx
+++ b/files/trading-journal-template.xlsx
@@ -115,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,6 +131,7 @@
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -205,6 +206,147 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Equity curve (cumulative R)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Journal'!L4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Journal'!$L$5:$L$204</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Trade #</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Cumulative R</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -510,6 +652,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -581,6 +724,11 @@
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Equity (R)</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -607,6 +755,10 @@
       </c>
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="6" t="n"/>
+      <c r="L5" s="7">
+        <f>IF(H5="","",SUM($H$5:H5))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -626,6 +778,10 @@
       </c>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
+      <c r="L6" s="7">
+        <f>IF(H6="","",SUM($H$5:H6))</f>
+        <v/>
+      </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
           <t>Total trades logged</t>
@@ -654,6 +810,10 @@
       </c>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
+      <c r="L7" s="7">
+        <f>IF(H7="","",SUM($H$5:H7))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -673,6 +833,10 @@
       </c>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
+      <c r="L8" s="7">
+        <f>IF(H8="","",SUM($H$5:H8))</f>
+        <v/>
+      </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
           <t>Win rate</t>
@@ -701,6 +865,10 @@
       </c>
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="6" t="n"/>
+      <c r="L9" s="7">
+        <f>IF(H9="","",SUM($H$5:H9))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -720,6 +888,10 @@
       </c>
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
+      <c r="L10" s="7">
+        <f>IF(H10="","",SUM($H$5:H10))</f>
+        <v/>
+      </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
           <t>Average R</t>
@@ -748,6 +920,10 @@
       </c>
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
+      <c r="L11" s="7">
+        <f>IF(H11="","",SUM($H$5:H11))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -767,6 +943,10 @@
       </c>
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
+      <c r="L12" s="7">
+        <f>IF(H12="","",SUM($H$5:H12))</f>
+        <v/>
+      </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
           <t>Average winner (R)</t>
@@ -795,6 +975,10 @@
       </c>
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
+      <c r="L13" s="7">
+        <f>IF(H13="","",SUM($H$5:H13))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -814,6 +998,10 @@
       </c>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
+      <c r="L14" s="7">
+        <f>IF(H14="","",SUM($H$5:H14))</f>
+        <v/>
+      </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
           <t>Average loser (R)</t>
@@ -842,6 +1030,10 @@
       </c>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
+      <c r="L15" s="7">
+        <f>IF(H15="","",SUM($H$5:H15))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -861,6 +1053,10 @@
       </c>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
+      <c r="L16" s="7">
+        <f>IF(H16="","",SUM($H$5:H16))</f>
+        <v/>
+      </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
           <t>Expectancy (R per trade)</t>
@@ -889,6 +1085,10 @@
       </c>
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
+      <c r="L17" s="7">
+        <f>IF(H17="","",SUM($H$5:H17))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -908,6 +1108,19 @@
       </c>
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
+      <c r="L18" s="7">
+        <f>IF(H18="","",SUM($H$5:H18))</f>
+        <v/>
+      </c>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>Largest winner (R)</t>
+        </is>
+      </c>
+      <c r="O18" s="11">
+        <f>IFERROR(MAXIFS(H5:H204,H5:H204,"&gt;0"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -927,6 +1140,10 @@
       </c>
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
+      <c r="L19" s="7">
+        <f>IF(H19="","",SUM($H$5:H19))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
@@ -946,6 +1163,19 @@
       </c>
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
+      <c r="L20" s="7">
+        <f>IF(H20="","",SUM($H$5:H20))</f>
+        <v/>
+      </c>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>Largest loser (R)</t>
+        </is>
+      </c>
+      <c r="O20" s="11">
+        <f>IFERROR(MINIFS(H5:H204,H5:H204,"&lt;0"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
@@ -965,6 +1195,10 @@
       </c>
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
+      <c r="L21" s="7">
+        <f>IF(H21="","",SUM($H$5:H21))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
@@ -984,6 +1218,19 @@
       </c>
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="6" t="n"/>
+      <c r="L22" s="7">
+        <f>IF(H22="","",SUM($H$5:H22))</f>
+        <v/>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>Profit factor</t>
+        </is>
+      </c>
+      <c r="O22" s="13">
+        <f>IFERROR(SUMIF(H5:H204,"&gt;0")/ABS(SUMIF(H5:H204,"&lt;0")),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1003,6 +1250,10 @@
       </c>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
+      <c r="L23" s="7">
+        <f>IF(H23="","",SUM($H$5:H23))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
@@ -1022,6 +1273,10 @@
       </c>
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="n"/>
+      <c r="L24" s="7">
+        <f>IF(H24="","",SUM($H$5:H24))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -1041,6 +1296,10 @@
       </c>
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n"/>
+      <c r="L25" s="7">
+        <f>IF(H25="","",SUM($H$5:H25))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
@@ -1060,6 +1319,10 @@
       </c>
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="n"/>
+      <c r="L26" s="7">
+        <f>IF(H26="","",SUM($H$5:H26))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
@@ -1079,6 +1342,10 @@
       </c>
       <c r="J27" s="6" t="n"/>
       <c r="K27" s="6" t="n"/>
+      <c r="L27" s="7">
+        <f>IF(H27="","",SUM($H$5:H27))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
@@ -1098,6 +1365,10 @@
       </c>
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="6" t="n"/>
+      <c r="L28" s="7">
+        <f>IF(H28="","",SUM($H$5:H28))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -1117,6 +1388,10 @@
       </c>
       <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="n"/>
+      <c r="L29" s="7">
+        <f>IF(H29="","",SUM($H$5:H29))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
@@ -1136,6 +1411,10 @@
       </c>
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="6" t="n"/>
+      <c r="L30" s="7">
+        <f>IF(H30="","",SUM($H$5:H30))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -1155,6 +1434,10 @@
       </c>
       <c r="J31" s="6" t="n"/>
       <c r="K31" s="6" t="n"/>
+      <c r="L31" s="7">
+        <f>IF(H31="","",SUM($H$5:H31))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
@@ -1174,6 +1457,10 @@
       </c>
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="n"/>
+      <c r="L32" s="7">
+        <f>IF(H32="","",SUM($H$5:H32))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -1193,6 +1480,10 @@
       </c>
       <c r="J33" s="6" t="n"/>
       <c r="K33" s="6" t="n"/>
+      <c r="L33" s="7">
+        <f>IF(H33="","",SUM($H$5:H33))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>
@@ -1212,6 +1503,10 @@
       </c>
       <c r="J34" s="6" t="n"/>
       <c r="K34" s="6" t="n"/>
+      <c r="L34" s="7">
+        <f>IF(H34="","",SUM($H$5:H34))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -1231,6 +1526,10 @@
       </c>
       <c r="J35" s="6" t="n"/>
       <c r="K35" s="6" t="n"/>
+      <c r="L35" s="7">
+        <f>IF(H35="","",SUM($H$5:H35))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n"/>
@@ -1250,6 +1549,10 @@
       </c>
       <c r="J36" s="6" t="n"/>
       <c r="K36" s="6" t="n"/>
+      <c r="L36" s="7">
+        <f>IF(H36="","",SUM($H$5:H36))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -1269,6 +1572,10 @@
       </c>
       <c r="J37" s="6" t="n"/>
       <c r="K37" s="6" t="n"/>
+      <c r="L37" s="7">
+        <f>IF(H37="","",SUM($H$5:H37))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
@@ -1288,6 +1595,10 @@
       </c>
       <c r="J38" s="6" t="n"/>
       <c r="K38" s="6" t="n"/>
+      <c r="L38" s="7">
+        <f>IF(H38="","",SUM($H$5:H38))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -1307,6 +1618,10 @@
       </c>
       <c r="J39" s="6" t="n"/>
       <c r="K39" s="6" t="n"/>
+      <c r="L39" s="7">
+        <f>IF(H39="","",SUM($H$5:H39))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n"/>
@@ -1326,6 +1641,10 @@
       </c>
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="6" t="n"/>
+      <c r="L40" s="7">
+        <f>IF(H40="","",SUM($H$5:H40))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -1345,6 +1664,10 @@
       </c>
       <c r="J41" s="6" t="n"/>
       <c r="K41" s="6" t="n"/>
+      <c r="L41" s="7">
+        <f>IF(H41="","",SUM($H$5:H41))</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
@@ -1364,6 +1687,10 @@
       </c>
       <c r="J42" s="6" t="n"/>
       <c r="K42" s="6" t="n"/>
+      <c r="L42" s="7">
+        <f>IF(H42="","",SUM($H$5:H42))</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -1383,6 +1710,10 @@
       </c>
       <c r="J43" s="6" t="n"/>
       <c r="K43" s="6" t="n"/>
+      <c r="L43" s="7">
+        <f>IF(H43="","",SUM($H$5:H43))</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
@@ -1402,6 +1733,10 @@
       </c>
       <c r="J44" s="6" t="n"/>
       <c r="K44" s="6" t="n"/>
+      <c r="L44" s="7">
+        <f>IF(H44="","",SUM($H$5:H44))</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -1421,6 +1756,10 @@
       </c>
       <c r="J45" s="6" t="n"/>
       <c r="K45" s="6" t="n"/>
+      <c r="L45" s="7">
+        <f>IF(H45="","",SUM($H$5:H45))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n"/>
@@ -1440,6 +1779,10 @@
       </c>
       <c r="J46" s="6" t="n"/>
       <c r="K46" s="6" t="n"/>
+      <c r="L46" s="7">
+        <f>IF(H46="","",SUM($H$5:H46))</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -1459,6 +1802,10 @@
       </c>
       <c r="J47" s="6" t="n"/>
       <c r="K47" s="6" t="n"/>
+      <c r="L47" s="7">
+        <f>IF(H47="","",SUM($H$5:H47))</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
@@ -1478,6 +1825,10 @@
       </c>
       <c r="J48" s="6" t="n"/>
       <c r="K48" s="6" t="n"/>
+      <c r="L48" s="7">
+        <f>IF(H48="","",SUM($H$5:H48))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -1497,6 +1848,10 @@
       </c>
       <c r="J49" s="6" t="n"/>
       <c r="K49" s="6" t="n"/>
+      <c r="L49" s="7">
+        <f>IF(H49="","",SUM($H$5:H49))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n"/>
@@ -1516,6 +1871,10 @@
       </c>
       <c r="J50" s="6" t="n"/>
       <c r="K50" s="6" t="n"/>
+      <c r="L50" s="7">
+        <f>IF(H50="","",SUM($H$5:H50))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -1535,6 +1894,10 @@
       </c>
       <c r="J51" s="6" t="n"/>
       <c r="K51" s="6" t="n"/>
+      <c r="L51" s="7">
+        <f>IF(H51="","",SUM($H$5:H51))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
@@ -1554,6 +1917,10 @@
       </c>
       <c r="J52" s="6" t="n"/>
       <c r="K52" s="6" t="n"/>
+      <c r="L52" s="7">
+        <f>IF(H52="","",SUM($H$5:H52))</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -1573,6 +1940,10 @@
       </c>
       <c r="J53" s="6" t="n"/>
       <c r="K53" s="6" t="n"/>
+      <c r="L53" s="7">
+        <f>IF(H53="","",SUM($H$5:H53))</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
@@ -1592,6 +1963,10 @@
       </c>
       <c r="J54" s="6" t="n"/>
       <c r="K54" s="6" t="n"/>
+      <c r="L54" s="7">
+        <f>IF(H54="","",SUM($H$5:H54))</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
@@ -1611,6 +1986,10 @@
       </c>
       <c r="J55" s="6" t="n"/>
       <c r="K55" s="6" t="n"/>
+      <c r="L55" s="7">
+        <f>IF(H55="","",SUM($H$5:H55))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n"/>
@@ -1630,6 +2009,10 @@
       </c>
       <c r="J56" s="6" t="n"/>
       <c r="K56" s="6" t="n"/>
+      <c r="L56" s="7">
+        <f>IF(H56="","",SUM($H$5:H56))</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
@@ -1649,6 +2032,10 @@
       </c>
       <c r="J57" s="6" t="n"/>
       <c r="K57" s="6" t="n"/>
+      <c r="L57" s="7">
+        <f>IF(H57="","",SUM($H$5:H57))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n"/>
@@ -1668,6 +2055,10 @@
       </c>
       <c r="J58" s="6" t="n"/>
       <c r="K58" s="6" t="n"/>
+      <c r="L58" s="7">
+        <f>IF(H58="","",SUM($H$5:H58))</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
@@ -1687,6 +2078,10 @@
       </c>
       <c r="J59" s="6" t="n"/>
       <c r="K59" s="6" t="n"/>
+      <c r="L59" s="7">
+        <f>IF(H59="","",SUM($H$5:H59))</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
@@ -1706,6 +2101,10 @@
       </c>
       <c r="J60" s="6" t="n"/>
       <c r="K60" s="6" t="n"/>
+      <c r="L60" s="7">
+        <f>IF(H60="","",SUM($H$5:H60))</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n"/>
@@ -1725,6 +2124,10 @@
       </c>
       <c r="J61" s="6" t="n"/>
       <c r="K61" s="6" t="n"/>
+      <c r="L61" s="7">
+        <f>IF(H61="","",SUM($H$5:H61))</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n"/>
@@ -1744,6 +2147,10 @@
       </c>
       <c r="J62" s="6" t="n"/>
       <c r="K62" s="6" t="n"/>
+      <c r="L62" s="7">
+        <f>IF(H62="","",SUM($H$5:H62))</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n"/>
@@ -1763,6 +2170,10 @@
       </c>
       <c r="J63" s="6" t="n"/>
       <c r="K63" s="6" t="n"/>
+      <c r="L63" s="7">
+        <f>IF(H63="","",SUM($H$5:H63))</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n"/>
@@ -1782,6 +2193,10 @@
       </c>
       <c r="J64" s="6" t="n"/>
       <c r="K64" s="6" t="n"/>
+      <c r="L64" s="7">
+        <f>IF(H64="","",SUM($H$5:H64))</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n"/>
@@ -1801,6 +2216,10 @@
       </c>
       <c r="J65" s="6" t="n"/>
       <c r="K65" s="6" t="n"/>
+      <c r="L65" s="7">
+        <f>IF(H65="","",SUM($H$5:H65))</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n"/>
@@ -1820,6 +2239,10 @@
       </c>
       <c r="J66" s="6" t="n"/>
       <c r="K66" s="6" t="n"/>
+      <c r="L66" s="7">
+        <f>IF(H66="","",SUM($H$5:H66))</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n"/>
@@ -1839,6 +2262,10 @@
       </c>
       <c r="J67" s="6" t="n"/>
       <c r="K67" s="6" t="n"/>
+      <c r="L67" s="7">
+        <f>IF(H67="","",SUM($H$5:H67))</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n"/>
@@ -1858,6 +2285,10 @@
       </c>
       <c r="J68" s="6" t="n"/>
       <c r="K68" s="6" t="n"/>
+      <c r="L68" s="7">
+        <f>IF(H68="","",SUM($H$5:H68))</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n"/>
@@ -1877,6 +2308,10 @@
       </c>
       <c r="J69" s="6" t="n"/>
       <c r="K69" s="6" t="n"/>
+      <c r="L69" s="7">
+        <f>IF(H69="","",SUM($H$5:H69))</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n"/>
@@ -1896,6 +2331,10 @@
       </c>
       <c r="J70" s="6" t="n"/>
       <c r="K70" s="6" t="n"/>
+      <c r="L70" s="7">
+        <f>IF(H70="","",SUM($H$5:H70))</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n"/>
@@ -1915,6 +2354,10 @@
       </c>
       <c r="J71" s="6" t="n"/>
       <c r="K71" s="6" t="n"/>
+      <c r="L71" s="7">
+        <f>IF(H71="","",SUM($H$5:H71))</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n"/>
@@ -1934,6 +2377,10 @@
       </c>
       <c r="J72" s="6" t="n"/>
       <c r="K72" s="6" t="n"/>
+      <c r="L72" s="7">
+        <f>IF(H72="","",SUM($H$5:H72))</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n"/>
@@ -1953,6 +2400,10 @@
       </c>
       <c r="J73" s="6" t="n"/>
       <c r="K73" s="6" t="n"/>
+      <c r="L73" s="7">
+        <f>IF(H73="","",SUM($H$5:H73))</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n"/>
@@ -1972,6 +2423,10 @@
       </c>
       <c r="J74" s="6" t="n"/>
       <c r="K74" s="6" t="n"/>
+      <c r="L74" s="7">
+        <f>IF(H74="","",SUM($H$5:H74))</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n"/>
@@ -1991,6 +2446,10 @@
       </c>
       <c r="J75" s="6" t="n"/>
       <c r="K75" s="6" t="n"/>
+      <c r="L75" s="7">
+        <f>IF(H75="","",SUM($H$5:H75))</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n"/>
@@ -2010,6 +2469,10 @@
       </c>
       <c r="J76" s="6" t="n"/>
       <c r="K76" s="6" t="n"/>
+      <c r="L76" s="7">
+        <f>IF(H76="","",SUM($H$5:H76))</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n"/>
@@ -2029,6 +2492,10 @@
       </c>
       <c r="J77" s="6" t="n"/>
       <c r="K77" s="6" t="n"/>
+      <c r="L77" s="7">
+        <f>IF(H77="","",SUM($H$5:H77))</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n"/>
@@ -2048,6 +2515,10 @@
       </c>
       <c r="J78" s="6" t="n"/>
       <c r="K78" s="6" t="n"/>
+      <c r="L78" s="7">
+        <f>IF(H78="","",SUM($H$5:H78))</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n"/>
@@ -2067,6 +2538,10 @@
       </c>
       <c r="J79" s="6" t="n"/>
       <c r="K79" s="6" t="n"/>
+      <c r="L79" s="7">
+        <f>IF(H79="","",SUM($H$5:H79))</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n"/>
@@ -2086,6 +2561,10 @@
       </c>
       <c r="J80" s="6" t="n"/>
       <c r="K80" s="6" t="n"/>
+      <c r="L80" s="7">
+        <f>IF(H80="","",SUM($H$5:H80))</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n"/>
@@ -2105,6 +2584,10 @@
       </c>
       <c r="J81" s="6" t="n"/>
       <c r="K81" s="6" t="n"/>
+      <c r="L81" s="7">
+        <f>IF(H81="","",SUM($H$5:H81))</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n"/>
@@ -2124,6 +2607,10 @@
       </c>
       <c r="J82" s="6" t="n"/>
       <c r="K82" s="6" t="n"/>
+      <c r="L82" s="7">
+        <f>IF(H82="","",SUM($H$5:H82))</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n"/>
@@ -2143,6 +2630,10 @@
       </c>
       <c r="J83" s="6" t="n"/>
       <c r="K83" s="6" t="n"/>
+      <c r="L83" s="7">
+        <f>IF(H83="","",SUM($H$5:H83))</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n"/>
@@ -2162,6 +2653,10 @@
       </c>
       <c r="J84" s="6" t="n"/>
       <c r="K84" s="6" t="n"/>
+      <c r="L84" s="7">
+        <f>IF(H84="","",SUM($H$5:H84))</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n"/>
@@ -2181,6 +2676,10 @@
       </c>
       <c r="J85" s="6" t="n"/>
       <c r="K85" s="6" t="n"/>
+      <c r="L85" s="7">
+        <f>IF(H85="","",SUM($H$5:H85))</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n"/>
@@ -2200,6 +2699,10 @@
       </c>
       <c r="J86" s="6" t="n"/>
       <c r="K86" s="6" t="n"/>
+      <c r="L86" s="7">
+        <f>IF(H86="","",SUM($H$5:H86))</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n"/>
@@ -2219,6 +2722,10 @@
       </c>
       <c r="J87" s="6" t="n"/>
       <c r="K87" s="6" t="n"/>
+      <c r="L87" s="7">
+        <f>IF(H87="","",SUM($H$5:H87))</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n"/>
@@ -2238,6 +2745,10 @@
       </c>
       <c r="J88" s="6" t="n"/>
       <c r="K88" s="6" t="n"/>
+      <c r="L88" s="7">
+        <f>IF(H88="","",SUM($H$5:H88))</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n"/>
@@ -2257,6 +2768,10 @@
       </c>
       <c r="J89" s="6" t="n"/>
       <c r="K89" s="6" t="n"/>
+      <c r="L89" s="7">
+        <f>IF(H89="","",SUM($H$5:H89))</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n"/>
@@ -2276,6 +2791,10 @@
       </c>
       <c r="J90" s="6" t="n"/>
       <c r="K90" s="6" t="n"/>
+      <c r="L90" s="7">
+        <f>IF(H90="","",SUM($H$5:H90))</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n"/>
@@ -2295,6 +2814,10 @@
       </c>
       <c r="J91" s="6" t="n"/>
       <c r="K91" s="6" t="n"/>
+      <c r="L91" s="7">
+        <f>IF(H91="","",SUM($H$5:H91))</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="n"/>
@@ -2314,6 +2837,10 @@
       </c>
       <c r="J92" s="6" t="n"/>
       <c r="K92" s="6" t="n"/>
+      <c r="L92" s="7">
+        <f>IF(H92="","",SUM($H$5:H92))</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="n"/>
@@ -2333,6 +2860,10 @@
       </c>
       <c r="J93" s="6" t="n"/>
       <c r="K93" s="6" t="n"/>
+      <c r="L93" s="7">
+        <f>IF(H93="","",SUM($H$5:H93))</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n"/>
@@ -2352,6 +2883,10 @@
       </c>
       <c r="J94" s="6" t="n"/>
       <c r="K94" s="6" t="n"/>
+      <c r="L94" s="7">
+        <f>IF(H94="","",SUM($H$5:H94))</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="n"/>
@@ -2371,6 +2906,10 @@
       </c>
       <c r="J95" s="6" t="n"/>
       <c r="K95" s="6" t="n"/>
+      <c r="L95" s="7">
+        <f>IF(H95="","",SUM($H$5:H95))</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n"/>
@@ -2390,6 +2929,10 @@
       </c>
       <c r="J96" s="6" t="n"/>
       <c r="K96" s="6" t="n"/>
+      <c r="L96" s="7">
+        <f>IF(H96="","",SUM($H$5:H96))</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n"/>
@@ -2409,6 +2952,10 @@
       </c>
       <c r="J97" s="6" t="n"/>
       <c r="K97" s="6" t="n"/>
+      <c r="L97" s="7">
+        <f>IF(H97="","",SUM($H$5:H97))</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n"/>
@@ -2428,6 +2975,10 @@
       </c>
       <c r="J98" s="6" t="n"/>
       <c r="K98" s="6" t="n"/>
+      <c r="L98" s="7">
+        <f>IF(H98="","",SUM($H$5:H98))</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="n"/>
@@ -2447,6 +2998,10 @@
       </c>
       <c r="J99" s="6" t="n"/>
       <c r="K99" s="6" t="n"/>
+      <c r="L99" s="7">
+        <f>IF(H99="","",SUM($H$5:H99))</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="n"/>
@@ -2466,6 +3021,10 @@
       </c>
       <c r="J100" s="6" t="n"/>
       <c r="K100" s="6" t="n"/>
+      <c r="L100" s="7">
+        <f>IF(H100="","",SUM($H$5:H100))</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="n"/>
@@ -2485,6 +3044,10 @@
       </c>
       <c r="J101" s="6" t="n"/>
       <c r="K101" s="6" t="n"/>
+      <c r="L101" s="7">
+        <f>IF(H101="","",SUM($H$5:H101))</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n"/>
@@ -2504,6 +3067,10 @@
       </c>
       <c r="J102" s="6" t="n"/>
       <c r="K102" s="6" t="n"/>
+      <c r="L102" s="7">
+        <f>IF(H102="","",SUM($H$5:H102))</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="n"/>
@@ -2523,6 +3090,10 @@
       </c>
       <c r="J103" s="6" t="n"/>
       <c r="K103" s="6" t="n"/>
+      <c r="L103" s="7">
+        <f>IF(H103="","",SUM($H$5:H103))</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n"/>
@@ -2542,6 +3113,10 @@
       </c>
       <c r="J104" s="6" t="n"/>
       <c r="K104" s="6" t="n"/>
+      <c r="L104" s="7">
+        <f>IF(H104="","",SUM($H$5:H104))</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="n"/>
@@ -2561,6 +3136,10 @@
       </c>
       <c r="J105" s="6" t="n"/>
       <c r="K105" s="6" t="n"/>
+      <c r="L105" s="7">
+        <f>IF(H105="","",SUM($H$5:H105))</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n"/>
@@ -2580,6 +3159,10 @@
       </c>
       <c r="J106" s="6" t="n"/>
       <c r="K106" s="6" t="n"/>
+      <c r="L106" s="7">
+        <f>IF(H106="","",SUM($H$5:H106))</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n"/>
@@ -2599,6 +3182,10 @@
       </c>
       <c r="J107" s="6" t="n"/>
       <c r="K107" s="6" t="n"/>
+      <c r="L107" s="7">
+        <f>IF(H107="","",SUM($H$5:H107))</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n"/>
@@ -2618,6 +3205,10 @@
       </c>
       <c r="J108" s="6" t="n"/>
       <c r="K108" s="6" t="n"/>
+      <c r="L108" s="7">
+        <f>IF(H108="","",SUM($H$5:H108))</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="n"/>
@@ -2637,6 +3228,10 @@
       </c>
       <c r="J109" s="6" t="n"/>
       <c r="K109" s="6" t="n"/>
+      <c r="L109" s="7">
+        <f>IF(H109="","",SUM($H$5:H109))</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n"/>
@@ -2656,6 +3251,10 @@
       </c>
       <c r="J110" s="6" t="n"/>
       <c r="K110" s="6" t="n"/>
+      <c r="L110" s="7">
+        <f>IF(H110="","",SUM($H$5:H110))</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n"/>
@@ -2675,6 +3274,10 @@
       </c>
       <c r="J111" s="6" t="n"/>
       <c r="K111" s="6" t="n"/>
+      <c r="L111" s="7">
+        <f>IF(H111="","",SUM($H$5:H111))</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="n"/>
@@ -2694,6 +3297,10 @@
       </c>
       <c r="J112" s="6" t="n"/>
       <c r="K112" s="6" t="n"/>
+      <c r="L112" s="7">
+        <f>IF(H112="","",SUM($H$5:H112))</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="n"/>
@@ -2713,6 +3320,10 @@
       </c>
       <c r="J113" s="6" t="n"/>
       <c r="K113" s="6" t="n"/>
+      <c r="L113" s="7">
+        <f>IF(H113="","",SUM($H$5:H113))</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="n"/>
@@ -2732,6 +3343,10 @@
       </c>
       <c r="J114" s="6" t="n"/>
       <c r="K114" s="6" t="n"/>
+      <c r="L114" s="7">
+        <f>IF(H114="","",SUM($H$5:H114))</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="n"/>
@@ -2751,6 +3366,10 @@
       </c>
       <c r="J115" s="6" t="n"/>
       <c r="K115" s="6" t="n"/>
+      <c r="L115" s="7">
+        <f>IF(H115="","",SUM($H$5:H115))</f>
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n"/>
@@ -2770,6 +3389,10 @@
       </c>
       <c r="J116" s="6" t="n"/>
       <c r="K116" s="6" t="n"/>
+      <c r="L116" s="7">
+        <f>IF(H116="","",SUM($H$5:H116))</f>
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="n"/>
@@ -2789,6 +3412,10 @@
       </c>
       <c r="J117" s="6" t="n"/>
       <c r="K117" s="6" t="n"/>
+      <c r="L117" s="7">
+        <f>IF(H117="","",SUM($H$5:H117))</f>
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="n"/>
@@ -2808,6 +3435,10 @@
       </c>
       <c r="J118" s="6" t="n"/>
       <c r="K118" s="6" t="n"/>
+      <c r="L118" s="7">
+        <f>IF(H118="","",SUM($H$5:H118))</f>
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n"/>
@@ -2827,6 +3458,10 @@
       </c>
       <c r="J119" s="6" t="n"/>
       <c r="K119" s="6" t="n"/>
+      <c r="L119" s="7">
+        <f>IF(H119="","",SUM($H$5:H119))</f>
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n"/>
@@ -2846,6 +3481,10 @@
       </c>
       <c r="J120" s="6" t="n"/>
       <c r="K120" s="6" t="n"/>
+      <c r="L120" s="7">
+        <f>IF(H120="","",SUM($H$5:H120))</f>
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n"/>
@@ -2865,6 +3504,10 @@
       </c>
       <c r="J121" s="6" t="n"/>
       <c r="K121" s="6" t="n"/>
+      <c r="L121" s="7">
+        <f>IF(H121="","",SUM($H$5:H121))</f>
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="n"/>
@@ -2884,6 +3527,10 @@
       </c>
       <c r="J122" s="6" t="n"/>
       <c r="K122" s="6" t="n"/>
+      <c r="L122" s="7">
+        <f>IF(H122="","",SUM($H$5:H122))</f>
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="n"/>
@@ -2903,6 +3550,10 @@
       </c>
       <c r="J123" s="6" t="n"/>
       <c r="K123" s="6" t="n"/>
+      <c r="L123" s="7">
+        <f>IF(H123="","",SUM($H$5:H123))</f>
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="n"/>
@@ -2922,6 +3573,10 @@
       </c>
       <c r="J124" s="6" t="n"/>
       <c r="K124" s="6" t="n"/>
+      <c r="L124" s="7">
+        <f>IF(H124="","",SUM($H$5:H124))</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="n"/>
@@ -2941,6 +3596,10 @@
       </c>
       <c r="J125" s="6" t="n"/>
       <c r="K125" s="6" t="n"/>
+      <c r="L125" s="7">
+        <f>IF(H125="","",SUM($H$5:H125))</f>
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="5" t="n"/>
@@ -2960,6 +3619,10 @@
       </c>
       <c r="J126" s="6" t="n"/>
       <c r="K126" s="6" t="n"/>
+      <c r="L126" s="7">
+        <f>IF(H126="","",SUM($H$5:H126))</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="n"/>
@@ -2979,6 +3642,10 @@
       </c>
       <c r="J127" s="6" t="n"/>
       <c r="K127" s="6" t="n"/>
+      <c r="L127" s="7">
+        <f>IF(H127="","",SUM($H$5:H127))</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="n"/>
@@ -2998,6 +3665,10 @@
       </c>
       <c r="J128" s="6" t="n"/>
       <c r="K128" s="6" t="n"/>
+      <c r="L128" s="7">
+        <f>IF(H128="","",SUM($H$5:H128))</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="n"/>
@@ -3017,6 +3688,10 @@
       </c>
       <c r="J129" s="6" t="n"/>
       <c r="K129" s="6" t="n"/>
+      <c r="L129" s="7">
+        <f>IF(H129="","",SUM($H$5:H129))</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n"/>
@@ -3036,6 +3711,10 @@
       </c>
       <c r="J130" s="6" t="n"/>
       <c r="K130" s="6" t="n"/>
+      <c r="L130" s="7">
+        <f>IF(H130="","",SUM($H$5:H130))</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="5" t="n"/>
@@ -3055,6 +3734,10 @@
       </c>
       <c r="J131" s="6" t="n"/>
       <c r="K131" s="6" t="n"/>
+      <c r="L131" s="7">
+        <f>IF(H131="","",SUM($H$5:H131))</f>
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="5" t="n"/>
@@ -3074,6 +3757,10 @@
       </c>
       <c r="J132" s="6" t="n"/>
       <c r="K132" s="6" t="n"/>
+      <c r="L132" s="7">
+        <f>IF(H132="","",SUM($H$5:H132))</f>
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="5" t="n"/>
@@ -3093,6 +3780,10 @@
       </c>
       <c r="J133" s="6" t="n"/>
       <c r="K133" s="6" t="n"/>
+      <c r="L133" s="7">
+        <f>IF(H133="","",SUM($H$5:H133))</f>
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="5" t="n"/>
@@ -3112,6 +3803,10 @@
       </c>
       <c r="J134" s="6" t="n"/>
       <c r="K134" s="6" t="n"/>
+      <c r="L134" s="7">
+        <f>IF(H134="","",SUM($H$5:H134))</f>
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="n"/>
@@ -3131,6 +3826,10 @@
       </c>
       <c r="J135" s="6" t="n"/>
       <c r="K135" s="6" t="n"/>
+      <c r="L135" s="7">
+        <f>IF(H135="","",SUM($H$5:H135))</f>
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n"/>
@@ -3150,6 +3849,10 @@
       </c>
       <c r="J136" s="6" t="n"/>
       <c r="K136" s="6" t="n"/>
+      <c r="L136" s="7">
+        <f>IF(H136="","",SUM($H$5:H136))</f>
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n"/>
@@ -3169,6 +3872,10 @@
       </c>
       <c r="J137" s="6" t="n"/>
       <c r="K137" s="6" t="n"/>
+      <c r="L137" s="7">
+        <f>IF(H137="","",SUM($H$5:H137))</f>
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="n"/>
@@ -3188,6 +3895,10 @@
       </c>
       <c r="J138" s="6" t="n"/>
       <c r="K138" s="6" t="n"/>
+      <c r="L138" s="7">
+        <f>IF(H138="","",SUM($H$5:H138))</f>
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="n"/>
@@ -3207,6 +3918,10 @@
       </c>
       <c r="J139" s="6" t="n"/>
       <c r="K139" s="6" t="n"/>
+      <c r="L139" s="7">
+        <f>IF(H139="","",SUM($H$5:H139))</f>
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="n"/>
@@ -3226,6 +3941,10 @@
       </c>
       <c r="J140" s="6" t="n"/>
       <c r="K140" s="6" t="n"/>
+      <c r="L140" s="7">
+        <f>IF(H140="","",SUM($H$5:H140))</f>
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="n"/>
@@ -3245,6 +3964,10 @@
       </c>
       <c r="J141" s="6" t="n"/>
       <c r="K141" s="6" t="n"/>
+      <c r="L141" s="7">
+        <f>IF(H141="","",SUM($H$5:H141))</f>
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="5" t="n"/>
@@ -3264,6 +3987,10 @@
       </c>
       <c r="J142" s="6" t="n"/>
       <c r="K142" s="6" t="n"/>
+      <c r="L142" s="7">
+        <f>IF(H142="","",SUM($H$5:H142))</f>
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="5" t="n"/>
@@ -3283,6 +4010,10 @@
       </c>
       <c r="J143" s="6" t="n"/>
       <c r="K143" s="6" t="n"/>
+      <c r="L143" s="7">
+        <f>IF(H143="","",SUM($H$5:H143))</f>
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n"/>
@@ -3302,6 +4033,10 @@
       </c>
       <c r="J144" s="6" t="n"/>
       <c r="K144" s="6" t="n"/>
+      <c r="L144" s="7">
+        <f>IF(H144="","",SUM($H$5:H144))</f>
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="n"/>
@@ -3321,6 +4056,10 @@
       </c>
       <c r="J145" s="6" t="n"/>
       <c r="K145" s="6" t="n"/>
+      <c r="L145" s="7">
+        <f>IF(H145="","",SUM($H$5:H145))</f>
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n"/>
@@ -3340,6 +4079,10 @@
       </c>
       <c r="J146" s="6" t="n"/>
       <c r="K146" s="6" t="n"/>
+      <c r="L146" s="7">
+        <f>IF(H146="","",SUM($H$5:H146))</f>
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n"/>
@@ -3359,6 +4102,10 @@
       </c>
       <c r="J147" s="6" t="n"/>
       <c r="K147" s="6" t="n"/>
+      <c r="L147" s="7">
+        <f>IF(H147="","",SUM($H$5:H147))</f>
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="5" t="n"/>
@@ -3378,6 +4125,10 @@
       </c>
       <c r="J148" s="6" t="n"/>
       <c r="K148" s="6" t="n"/>
+      <c r="L148" s="7">
+        <f>IF(H148="","",SUM($H$5:H148))</f>
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="n"/>
@@ -3397,6 +4148,10 @@
       </c>
       <c r="J149" s="6" t="n"/>
       <c r="K149" s="6" t="n"/>
+      <c r="L149" s="7">
+        <f>IF(H149="","",SUM($H$5:H149))</f>
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="5" t="n"/>
@@ -3416,6 +4171,10 @@
       </c>
       <c r="J150" s="6" t="n"/>
       <c r="K150" s="6" t="n"/>
+      <c r="L150" s="7">
+        <f>IF(H150="","",SUM($H$5:H150))</f>
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="5" t="n"/>
@@ -3435,6 +4194,10 @@
       </c>
       <c r="J151" s="6" t="n"/>
       <c r="K151" s="6" t="n"/>
+      <c r="L151" s="7">
+        <f>IF(H151="","",SUM($H$5:H151))</f>
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="5" t="n"/>
@@ -3454,6 +4217,10 @@
       </c>
       <c r="J152" s="6" t="n"/>
       <c r="K152" s="6" t="n"/>
+      <c r="L152" s="7">
+        <f>IF(H152="","",SUM($H$5:H152))</f>
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="n"/>
@@ -3473,6 +4240,10 @@
       </c>
       <c r="J153" s="6" t="n"/>
       <c r="K153" s="6" t="n"/>
+      <c r="L153" s="7">
+        <f>IF(H153="","",SUM($H$5:H153))</f>
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="5" t="n"/>
@@ -3492,6 +4263,10 @@
       </c>
       <c r="J154" s="6" t="n"/>
       <c r="K154" s="6" t="n"/>
+      <c r="L154" s="7">
+        <f>IF(H154="","",SUM($H$5:H154))</f>
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="n"/>
@@ -3511,6 +4286,10 @@
       </c>
       <c r="J155" s="6" t="n"/>
       <c r="K155" s="6" t="n"/>
+      <c r="L155" s="7">
+        <f>IF(H155="","",SUM($H$5:H155))</f>
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n"/>
@@ -3530,6 +4309,10 @@
       </c>
       <c r="J156" s="6" t="n"/>
       <c r="K156" s="6" t="n"/>
+      <c r="L156" s="7">
+        <f>IF(H156="","",SUM($H$5:H156))</f>
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="n"/>
@@ -3549,6 +4332,10 @@
       </c>
       <c r="J157" s="6" t="n"/>
       <c r="K157" s="6" t="n"/>
+      <c r="L157" s="7">
+        <f>IF(H157="","",SUM($H$5:H157))</f>
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="5" t="n"/>
@@ -3568,6 +4355,10 @@
       </c>
       <c r="J158" s="6" t="n"/>
       <c r="K158" s="6" t="n"/>
+      <c r="L158" s="7">
+        <f>IF(H158="","",SUM($H$5:H158))</f>
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="5" t="n"/>
@@ -3587,6 +4378,10 @@
       </c>
       <c r="J159" s="6" t="n"/>
       <c r="K159" s="6" t="n"/>
+      <c r="L159" s="7">
+        <f>IF(H159="","",SUM($H$5:H159))</f>
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="5" t="n"/>
@@ -3606,6 +4401,10 @@
       </c>
       <c r="J160" s="6" t="n"/>
       <c r="K160" s="6" t="n"/>
+      <c r="L160" s="7">
+        <f>IF(H160="","",SUM($H$5:H160))</f>
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="5" t="n"/>
@@ -3625,6 +4424,10 @@
       </c>
       <c r="J161" s="6" t="n"/>
       <c r="K161" s="6" t="n"/>
+      <c r="L161" s="7">
+        <f>IF(H161="","",SUM($H$5:H161))</f>
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="5" t="n"/>
@@ -3644,6 +4447,10 @@
       </c>
       <c r="J162" s="6" t="n"/>
       <c r="K162" s="6" t="n"/>
+      <c r="L162" s="7">
+        <f>IF(H162="","",SUM($H$5:H162))</f>
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="n"/>
@@ -3663,6 +4470,10 @@
       </c>
       <c r="J163" s="6" t="n"/>
       <c r="K163" s="6" t="n"/>
+      <c r="L163" s="7">
+        <f>IF(H163="","",SUM($H$5:H163))</f>
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="5" t="n"/>
@@ -3682,6 +4493,10 @@
       </c>
       <c r="J164" s="6" t="n"/>
       <c r="K164" s="6" t="n"/>
+      <c r="L164" s="7">
+        <f>IF(H164="","",SUM($H$5:H164))</f>
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="n"/>
@@ -3701,6 +4516,10 @@
       </c>
       <c r="J165" s="6" t="n"/>
       <c r="K165" s="6" t="n"/>
+      <c r="L165" s="7">
+        <f>IF(H165="","",SUM($H$5:H165))</f>
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="5" t="n"/>
@@ -3720,6 +4539,10 @@
       </c>
       <c r="J166" s="6" t="n"/>
       <c r="K166" s="6" t="n"/>
+      <c r="L166" s="7">
+        <f>IF(H166="","",SUM($H$5:H166))</f>
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="5" t="n"/>
@@ -3739,6 +4562,10 @@
       </c>
       <c r="J167" s="6" t="n"/>
       <c r="K167" s="6" t="n"/>
+      <c r="L167" s="7">
+        <f>IF(H167="","",SUM($H$5:H167))</f>
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="5" t="n"/>
@@ -3758,6 +4585,10 @@
       </c>
       <c r="J168" s="6" t="n"/>
       <c r="K168" s="6" t="n"/>
+      <c r="L168" s="7">
+        <f>IF(H168="","",SUM($H$5:H168))</f>
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="5" t="n"/>
@@ -3777,6 +4608,10 @@
       </c>
       <c r="J169" s="6" t="n"/>
       <c r="K169" s="6" t="n"/>
+      <c r="L169" s="7">
+        <f>IF(H169="","",SUM($H$5:H169))</f>
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="5" t="n"/>
@@ -3796,6 +4631,10 @@
       </c>
       <c r="J170" s="6" t="n"/>
       <c r="K170" s="6" t="n"/>
+      <c r="L170" s="7">
+        <f>IF(H170="","",SUM($H$5:H170))</f>
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="5" t="n"/>
@@ -3815,6 +4654,10 @@
       </c>
       <c r="J171" s="6" t="n"/>
       <c r="K171" s="6" t="n"/>
+      <c r="L171" s="7">
+        <f>IF(H171="","",SUM($H$5:H171))</f>
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="5" t="n"/>
@@ -3834,6 +4677,10 @@
       </c>
       <c r="J172" s="6" t="n"/>
       <c r="K172" s="6" t="n"/>
+      <c r="L172" s="7">
+        <f>IF(H172="","",SUM($H$5:H172))</f>
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="5" t="n"/>
@@ -3853,6 +4700,10 @@
       </c>
       <c r="J173" s="6" t="n"/>
       <c r="K173" s="6" t="n"/>
+      <c r="L173" s="7">
+        <f>IF(H173="","",SUM($H$5:H173))</f>
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="5" t="n"/>
@@ -3872,6 +4723,10 @@
       </c>
       <c r="J174" s="6" t="n"/>
       <c r="K174" s="6" t="n"/>
+      <c r="L174" s="7">
+        <f>IF(H174="","",SUM($H$5:H174))</f>
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="5" t="n"/>
@@ -3891,6 +4746,10 @@
       </c>
       <c r="J175" s="6" t="n"/>
       <c r="K175" s="6" t="n"/>
+      <c r="L175" s="7">
+        <f>IF(H175="","",SUM($H$5:H175))</f>
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="5" t="n"/>
@@ -3910,6 +4769,10 @@
       </c>
       <c r="J176" s="6" t="n"/>
       <c r="K176" s="6" t="n"/>
+      <c r="L176" s="7">
+        <f>IF(H176="","",SUM($H$5:H176))</f>
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="5" t="n"/>
@@ -3929,6 +4792,10 @@
       </c>
       <c r="J177" s="6" t="n"/>
       <c r="K177" s="6" t="n"/>
+      <c r="L177" s="7">
+        <f>IF(H177="","",SUM($H$5:H177))</f>
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n"/>
@@ -3948,6 +4815,10 @@
       </c>
       <c r="J178" s="6" t="n"/>
       <c r="K178" s="6" t="n"/>
+      <c r="L178" s="7">
+        <f>IF(H178="","",SUM($H$5:H178))</f>
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="5" t="n"/>
@@ -3967,6 +4838,10 @@
       </c>
       <c r="J179" s="6" t="n"/>
       <c r="K179" s="6" t="n"/>
+      <c r="L179" s="7">
+        <f>IF(H179="","",SUM($H$5:H179))</f>
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="5" t="n"/>
@@ -3986,6 +4861,10 @@
       </c>
       <c r="J180" s="6" t="n"/>
       <c r="K180" s="6" t="n"/>
+      <c r="L180" s="7">
+        <f>IF(H180="","",SUM($H$5:H180))</f>
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="5" t="n"/>
@@ -4005,6 +4884,10 @@
       </c>
       <c r="J181" s="6" t="n"/>
       <c r="K181" s="6" t="n"/>
+      <c r="L181" s="7">
+        <f>IF(H181="","",SUM($H$5:H181))</f>
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n"/>
@@ -4024,6 +4907,10 @@
       </c>
       <c r="J182" s="6" t="n"/>
       <c r="K182" s="6" t="n"/>
+      <c r="L182" s="7">
+        <f>IF(H182="","",SUM($H$5:H182))</f>
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n"/>
@@ -4043,6 +4930,10 @@
       </c>
       <c r="J183" s="6" t="n"/>
       <c r="K183" s="6" t="n"/>
+      <c r="L183" s="7">
+        <f>IF(H183="","",SUM($H$5:H183))</f>
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="5" t="n"/>
@@ -4062,6 +4953,10 @@
       </c>
       <c r="J184" s="6" t="n"/>
       <c r="K184" s="6" t="n"/>
+      <c r="L184" s="7">
+        <f>IF(H184="","",SUM($H$5:H184))</f>
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="5" t="n"/>
@@ -4081,6 +4976,10 @@
       </c>
       <c r="J185" s="6" t="n"/>
       <c r="K185" s="6" t="n"/>
+      <c r="L185" s="7">
+        <f>IF(H185="","",SUM($H$5:H185))</f>
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n"/>
@@ -4100,6 +4999,10 @@
       </c>
       <c r="J186" s="6" t="n"/>
       <c r="K186" s="6" t="n"/>
+      <c r="L186" s="7">
+        <f>IF(H186="","",SUM($H$5:H186))</f>
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n"/>
@@ -4119,6 +5022,10 @@
       </c>
       <c r="J187" s="6" t="n"/>
       <c r="K187" s="6" t="n"/>
+      <c r="L187" s="7">
+        <f>IF(H187="","",SUM($H$5:H187))</f>
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n"/>
@@ -4138,6 +5045,10 @@
       </c>
       <c r="J188" s="6" t="n"/>
       <c r="K188" s="6" t="n"/>
+      <c r="L188" s="7">
+        <f>IF(H188="","",SUM($H$5:H188))</f>
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n"/>
@@ -4157,6 +5068,10 @@
       </c>
       <c r="J189" s="6" t="n"/>
       <c r="K189" s="6" t="n"/>
+      <c r="L189" s="7">
+        <f>IF(H189="","",SUM($H$5:H189))</f>
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n"/>
@@ -4176,6 +5091,10 @@
       </c>
       <c r="J190" s="6" t="n"/>
       <c r="K190" s="6" t="n"/>
+      <c r="L190" s="7">
+        <f>IF(H190="","",SUM($H$5:H190))</f>
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="5" t="n"/>
@@ -4195,6 +5114,10 @@
       </c>
       <c r="J191" s="6" t="n"/>
       <c r="K191" s="6" t="n"/>
+      <c r="L191" s="7">
+        <f>IF(H191="","",SUM($H$5:H191))</f>
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="5" t="n"/>
@@ -4214,6 +5137,10 @@
       </c>
       <c r="J192" s="6" t="n"/>
       <c r="K192" s="6" t="n"/>
+      <c r="L192" s="7">
+        <f>IF(H192="","",SUM($H$5:H192))</f>
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n"/>
@@ -4233,6 +5160,10 @@
       </c>
       <c r="J193" s="6" t="n"/>
       <c r="K193" s="6" t="n"/>
+      <c r="L193" s="7">
+        <f>IF(H193="","",SUM($H$5:H193))</f>
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n"/>
@@ -4252,6 +5183,10 @@
       </c>
       <c r="J194" s="6" t="n"/>
       <c r="K194" s="6" t="n"/>
+      <c r="L194" s="7">
+        <f>IF(H194="","",SUM($H$5:H194))</f>
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="5" t="n"/>
@@ -4271,6 +5206,10 @@
       </c>
       <c r="J195" s="6" t="n"/>
       <c r="K195" s="6" t="n"/>
+      <c r="L195" s="7">
+        <f>IF(H195="","",SUM($H$5:H195))</f>
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="5" t="n"/>
@@ -4290,6 +5229,10 @@
       </c>
       <c r="J196" s="6" t="n"/>
       <c r="K196" s="6" t="n"/>
+      <c r="L196" s="7">
+        <f>IF(H196="","",SUM($H$5:H196))</f>
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n"/>
@@ -4309,6 +5252,10 @@
       </c>
       <c r="J197" s="6" t="n"/>
       <c r="K197" s="6" t="n"/>
+      <c r="L197" s="7">
+        <f>IF(H197="","",SUM($H$5:H197))</f>
+        <v/>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="5" t="n"/>
@@ -4328,6 +5275,10 @@
       </c>
       <c r="J198" s="6" t="n"/>
       <c r="K198" s="6" t="n"/>
+      <c r="L198" s="7">
+        <f>IF(H198="","",SUM($H$5:H198))</f>
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n"/>
@@ -4347,6 +5298,10 @@
       </c>
       <c r="J199" s="6" t="n"/>
       <c r="K199" s="6" t="n"/>
+      <c r="L199" s="7">
+        <f>IF(H199="","",SUM($H$5:H199))</f>
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n"/>
@@ -4366,6 +5321,10 @@
       </c>
       <c r="J200" s="6" t="n"/>
       <c r="K200" s="6" t="n"/>
+      <c r="L200" s="7">
+        <f>IF(H200="","",SUM($H$5:H200))</f>
+        <v/>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="5" t="n"/>
@@ -4385,6 +5344,10 @@
       </c>
       <c r="J201" s="6" t="n"/>
       <c r="K201" s="6" t="n"/>
+      <c r="L201" s="7">
+        <f>IF(H201="","",SUM($H$5:H201))</f>
+        <v/>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="5" t="n"/>
@@ -4404,6 +5367,10 @@
       </c>
       <c r="J202" s="6" t="n"/>
       <c r="K202" s="6" t="n"/>
+      <c r="L202" s="7">
+        <f>IF(H202="","",SUM($H$5:H202))</f>
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="5" t="n"/>
@@ -4423,6 +5390,10 @@
       </c>
       <c r="J203" s="6" t="n"/>
       <c r="K203" s="6" t="n"/>
+      <c r="L203" s="7">
+        <f>IF(H203="","",SUM($H$5:H203))</f>
+        <v/>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="5" t="n"/>
@@ -4442,6 +5413,10 @@
       </c>
       <c r="J204" s="6" t="n"/>
       <c r="K204" s="6" t="n"/>
+      <c r="L204" s="7">
+        <f>IF(H204="","",SUM($H$5:H204))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4457,5 +5432,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>